<commit_message>
Update Leaderboard and Pod
</commit_message>
<xml_diff>
--- a/public/tamplate_excel/data_courier.xlsx
+++ b/public/tamplate_excel/data_courier.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11060" tabRatio="500"/>
+    <workbookView windowHeight="17160" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="All Master Data Kurir" sheetId="3" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>id kurir</t>
   </si>
@@ -47,12 +47,15 @@
     <t>Area</t>
   </si>
   <si>
+    <t>Zona Delivery</t>
+  </si>
+  <si>
+    <t>no tlp (diawali 62)</t>
+  </si>
+  <si>
     <t>Zona</t>
   </si>
   <si>
-    <t>no tlp (diawali 62)</t>
-  </si>
-  <si>
     <t>BDO123</t>
   </si>
   <si>
@@ -75,6 +78,9 @@
   </si>
   <si>
     <t>6281212101212</t>
+  </si>
+  <si>
+    <t>BDO014</t>
   </si>
 </sst>
 </file>
@@ -708,11 +714,14 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -1048,8 +1057,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="1" outlineLevelCol="7"/>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="16.6328125" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
@@ -1057,7 +1066,7 @@
     <col min="4" max="4" width="16.09375" customWidth="1"/>
     <col min="5" max="5" width="25.3671875" customWidth="1"/>
     <col min="6" max="6" width="24.453125" customWidth="1"/>
-    <col min="7" max="7" width="8.1796875" customWidth="1"/>
+    <col min="7" max="7" width="12.4375" customWidth="1"/>
     <col min="8" max="8" width="15.7265625" customWidth="1"/>
     <col min="9" max="9" width="15.1796875" customWidth="1"/>
     <col min="10" max="10" width="17.3671875" customWidth="1"/>
@@ -1065,7 +1074,7 @@
     <col min="12" max="12" width="13.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1090,31 +1099,37 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:9">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="C2" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="4" t="s">
         <v>15</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>